<commit_message>
feat(F-NAR-019): TREE-AUT-005 polish Le coq et les bottes de Raphaël
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-005.xlsx
+++ b/stories/arbres/TREE-AUT-005.xlsx
@@ -854,7 +854,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Après la pluie, à la ferme, le volet bleu tape toc. Le coq a chanté une fois derrière la grange, puis s'est tu. Raphaël veut le rejoindre tout de suite, ballon, seau de grain ou doudou à la main. Pieds nus, la pierre mouillée le pique : il met la botte gauche, puis la droite. Sur le chemin, chat, chien ou poule font autre chose que prévu. La première idée rate. L'animal montre trois coins : le secret du cabanon, le fournil, les tomates. Raphaël comprend sans forcer le coq. Le toc du loquet paie le volet. Les bottes gardent boue et paille.</t>
+          <t>Après la pluie, à la ferme, le volet bleu tape toc. Le coq a chanté une fois derrière la grange, puis s'est tu. Raphaël veut le rejoindre vite, ballon, seau de grain ou doudou à la main. Pieds nus, la pierre mouillée le pique : il met la botte gauche, puis la droite. Sur le chemin, chat, chien ou poule font autre chose que prévu. La première idée rate. L'animal montre trois coins : le secret du cabanon, le fournil, les tomates. Raphaël comprend sans forcer le coq. Le toc du loquet paie le volet. Les bottes gardent boue et paille.</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>les bottes | bottes | ses bottes | les bottes d'abord | mettre les bottes</t>
+          <t>les bottes | bottes | ses bottes | les bottes d'abord | mettre les bottes | les bottes de Raphaël</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -2577,7 +2577,7 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>le secret du cabanon</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>après la sieste</t>
+          <t>le fournil</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>les tomates</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -3123,17 +3123,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Le fournil sent le pain, tout chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le coq est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
+          <t>Le fournil sent le pain, bien chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le coq est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil sent le pain, tout chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil sent le pain, bien chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Le fournil sent le pain, tout chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
+          <t>Le fournil sent le pain, bien chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>narrateur|Le fournil sent le pain, tout chaud.
+          <t>narrateur|Le fournil sent le pain, bien chaud.
 narrateur|De la farine flotte, blanche, légère.
 narrateur|Le chat éternue, et saute d'un sac.
 enfant-m|Le coq est sur la planche !
@@ -4100,7 +4100,7 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>le secret du cabanon</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>après la sieste</t>
+          <t>le fournil</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>les tomates</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -5622,7 +5622,7 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>le secret du cabanon</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -5632,7 +5632,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>après la sieste</t>
+          <t>le fournil</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>les tomates</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
@@ -6168,17 +6168,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le coq cligne. Il se ferme, tout petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
+          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le coq cligne. Il se ferme, très petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, tout petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, très petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, tout petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
+          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, très petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le ballon rouge sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6317,7 +6317,7 @@
 enfant-m|Coq, viens, c'est bon ici !
 narrateur|Raphaël tape des mains, trop fort.
 narrateur|La farine saute, et le coq cligne.
-enfant-m|Il se ferme, tout petit.
+enfant-m|Il se ferme, très petit.
 maman|Plus de mains, la pierre suffit.
 narrateur|La poule picore, sans bruit, maintenant.
 narrateur|Le coq baisse une aile, moins dur.
@@ -7136,7 +7136,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>les bottes | bottes | ses bottes | les bottes d'abord | mettre les bottes</t>
+          <t>les bottes | bottes | ses bottes | les bottes d'abord | mettre les bottes | les bottes de Raphaël</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -7905,7 +7905,7 @@
       <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>le secret du cabanon</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -7915,7 +7915,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>après la sieste</t>
+          <t>le fournil</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -7925,7 +7925,7 @@
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>les tomates</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
@@ -8451,17 +8451,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Le fournil sent le pain, tout chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le coq est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
+          <t>Le fournil sent le pain, bien chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le coq est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil sent le pain, tout chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil sent le pain, bien chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Le fournil sent le pain, tout chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
+          <t>Le fournil sent le pain, bien chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8595,7 +8595,7 @@
       </c>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>narrateur|Le fournil sent le pain, tout chaud.
+          <t>narrateur|Le fournil sent le pain, bien chaud.
 narrateur|De la farine flotte, blanche, légère.
 narrateur|Le chat éternue, et saute d'un sac.
 enfant-m|Le coq est sur la planche !
@@ -9428,7 +9428,7 @@
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>le secret du cabanon</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>après la sieste</t>
+          <t>le fournil</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>les tomates</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
@@ -10950,7 +10950,7 @@
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>le secret du cabanon</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>après la sieste</t>
+          <t>le fournil</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -10970,7 +10970,7 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>les tomates</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr">
@@ -11496,17 +11496,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le coq cligne. Il se ferme, tout petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
+          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le coq cligne. Il se ferme, très petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, tout petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, très petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, tout petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
+          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, très petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le seau bleu sur la pierre tiède. Le dernier grain sonne, tout petit. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11645,7 +11645,7 @@
 enfant-m|Coq, viens, c'est bon ici !
 narrateur|Raphaël tape des mains, trop fort.
 narrateur|La farine saute, et le coq cligne.
-enfant-m|Il se ferme, tout petit.
+enfant-m|Il se ferme, très petit.
 maman|Plus de mains, la pierre suffit.
 narrateur|La poule picore, sans bruit, maintenant.
 narrateur|Le coq baisse une aile, moins dur.
@@ -12464,7 +12464,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>les bottes | bottes | ses bottes | les bottes d'abord | mettre les bottes</t>
+          <t>les bottes | bottes | ses bottes | les bottes d'abord | mettre les bottes | les bottes de Raphaël</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -13236,7 +13236,7 @@
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>le secret du cabanon</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -13246,7 +13246,7 @@
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>après la sieste</t>
+          <t>le fournil</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">
@@ -13256,7 +13256,7 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>les tomates</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
@@ -13782,17 +13782,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Le fournil sent le pain, tout chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le coq est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
+          <t>Le fournil sent le pain, bien chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le coq est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil sent le pain, tout chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil sent le pain, bien chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Le fournil sent le pain, tout chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
+          <t>Le fournil sent le pain, bien chaud. De la farine flotte, blanche, légère. Le chat éternue, et saute d'un sac. Le &lt;emphasis&gt;coq&lt;/emphasis&gt; est sur la planche ! Raphaël tape des mains, pour l'appeler. Un nuage blanc cache tout, un moment. Je ne le vois plus. Plus de bruit, laisse la farine tomber. Le coq est là, plumes blanches. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13926,7 +13926,7 @@
       </c>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>narrateur|Le fournil sent le pain, tout chaud.
+          <t>narrateur|Le fournil sent le pain, bien chaud.
 narrateur|De la farine flotte, blanche, légère.
 narrateur|Le chat éternue, et saute d'un sac.
 enfant-m|Le coq est sur la planche !
@@ -14758,7 +14758,7 @@
       <c r="L73" s="2" t="inlineStr"/>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>le secret du cabanon</t>
         </is>
       </c>
       <c r="N73" s="2" t="inlineStr">
@@ -14768,7 +14768,7 @@
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>après la sieste</t>
+          <t>le fournil</t>
         </is>
       </c>
       <c r="P73" s="2" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="Q73" s="2" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>les tomates</t>
         </is>
       </c>
       <c r="R73" s="2" t="inlineStr">
@@ -16279,7 +16279,7 @@
       <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>le secret du cabanon</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
@@ -16289,7 +16289,7 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>après la sieste</t>
+          <t>le fournil</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
@@ -16299,7 +16299,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>les tomates</t>
         </is>
       </c>
       <c r="R81" s="2" t="inlineStr">
@@ -16825,17 +16825,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le coq cligne. Il se ferme, tout petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
+          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le coq cligne. Il se ferme, très petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, tout petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis level="moderate"&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, très petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, tout petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
+          <t>Le fournil a une pierre tiède, au bord. La poule picore la farine, chh. Coq, viens, c'est bon ici ! Raphaël tape des mains, trop fort. La farine saute, et le &lt;emphasis&gt;coq&lt;/emphasis&gt; cligne. Il se ferme, très petit. Plus de mains, la pierre suffit. La poule picore, sans bruit, maintenant. Le coq baisse une aile, moins dur. Raphaël pose le doudou sur la pierre. Un peu de grain, s'il en reste. Je ne te prends pas. Le coq descend, une patte, puis l'autre. La vapeur ressemble au lait du bol. Il est venu, tout seul. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16974,7 +16974,7 @@
 enfant-m|Coq, viens, c'est bon ici !
 narrateur|Raphaël tape des mains, trop fort.
 narrateur|La farine saute, et le coq cligne.
-enfant-m|Il se ferme, tout petit.
+enfant-m|Il se ferme, très petit.
 maman|Plus de mains, la pierre suffit.
 narrateur|La poule picore, sans bruit, maintenant.
 narrateur|Le coq baisse une aile, moins dur.
@@ -17575,7 +17575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17653,6 +17653,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>